<commit_message>
fix issue with country matching in GPT-4o base new30 answers
</commit_message>
<xml_diff>
--- a/eval/error_analysis/results/analysis_by_qid_full150.xlsx
+++ b/eval/error_analysis/results/analysis_by_qid_full150.xlsx
@@ -20509,7 +20509,7 @@
         </is>
       </c>
       <c r="P95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q95" t="inlineStr">
         <is>
@@ -28595,7 +28595,7 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K46" t="inlineStr">
         <is>
@@ -29909,7 +29909,7 @@
         </is>
       </c>
       <c r="J63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -29941,7 +29941,7 @@
         </is>
       </c>
       <c r="R63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S63" t="inlineStr">
         <is>
@@ -32389,7 +32389,7 @@
         </is>
       </c>
       <c r="J95" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K95" t="inlineStr">
         <is>
@@ -33333,7 +33333,7 @@
         </is>
       </c>
       <c r="J107" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K107" t="inlineStr">
         <is>
@@ -34577,7 +34577,7 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="n">
@@ -35564,7 +35564,7 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G136" t="inlineStr">
         <is>
@@ -36296,7 +36296,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix new30 verbose incorrect issues
</commit_message>
<xml_diff>
--- a/eval/error_analysis/results/analysis_by_qid_full150.xlsx
+++ b/eval/error_analysis/results/analysis_by_qid_full150.xlsx
@@ -24029,7 +24029,7 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
@@ -30131,7 +30131,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -33849,7 +33849,7 @@
         </is>
       </c>
       <c r="R113" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S113" t="inlineStr">
         <is>
@@ -34866,7 +34866,7 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G127" t="inlineStr"/>
       <c r="H127" t="n">
@@ -35174,7 +35174,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -35182,7 +35182,7 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
@@ -35190,7 +35190,7 @@
         </is>
       </c>
       <c r="H131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I131" t="inlineStr">
         <is>
@@ -35198,7 +35198,7 @@
         </is>
       </c>
       <c r="J131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K131" t="inlineStr">
         <is>
@@ -35206,7 +35206,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M131" t="inlineStr">
         <is>
@@ -35214,7 +35214,7 @@
         </is>
       </c>
       <c r="N131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O131" t="inlineStr">
         <is>
@@ -35222,7 +35222,7 @@
         </is>
       </c>
       <c r="P131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
@@ -35230,7 +35230,7 @@
         </is>
       </c>
       <c r="R131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S131" t="inlineStr">
         <is>
@@ -35238,7 +35238,7 @@
         </is>
       </c>
       <c r="T131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132">
@@ -35942,7 +35942,7 @@
         </is>
       </c>
       <c r="H141" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I141" t="inlineStr">
         <is>
@@ -35950,7 +35950,7 @@
         </is>
       </c>
       <c r="J141" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K141" t="inlineStr">
         <is>
@@ -35958,7 +35958,7 @@
         </is>
       </c>
       <c r="L141" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M141" t="inlineStr">
         <is>
@@ -35966,7 +35966,7 @@
         </is>
       </c>
       <c r="N141" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O141" t="inlineStr">
         <is>
@@ -35982,7 +35982,7 @@
         </is>
       </c>
       <c r="R141" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S141" t="inlineStr">
         <is>
@@ -35990,7 +35990,7 @@
         </is>
       </c>
       <c r="T141" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="142">
@@ -36242,7 +36242,7 @@
         </is>
       </c>
       <c r="F145" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G145" t="inlineStr"/>
       <c r="H145" t="n">
@@ -36440,7 +36440,7 @@
         </is>
       </c>
       <c r="F148" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G148" t="inlineStr"/>
       <c r="H148" t="n">
@@ -36580,7 +36580,7 @@
         </is>
       </c>
       <c r="F150" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
@@ -36650,7 +36650,7 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix partial match logic
</commit_message>
<xml_diff>
--- a/eval/error_analysis/results/analysis_by_qid_full150.xlsx
+++ b/eval/error_analysis/results/analysis_by_qid_full150.xlsx
@@ -13137,7 +13137,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -13219,7 +13219,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -13817,7 +13817,7 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -14309,7 +14309,7 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -16081,7 +16081,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -16679,7 +16679,7 @@
         </is>
       </c>
       <c r="P48" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
@@ -17221,7 +17221,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
@@ -17269,7 +17269,7 @@
         </is>
       </c>
       <c r="T55" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
@@ -17467,7 +17467,7 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I58" t="inlineStr">
         <is>
@@ -17491,7 +17491,7 @@
         </is>
       </c>
       <c r="N58" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
@@ -18443,7 +18443,7 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
@@ -18467,7 +18467,7 @@
         </is>
       </c>
       <c r="N70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
@@ -18491,7 +18491,7 @@
         </is>
       </c>
       <c r="T70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="71">
@@ -18627,7 +18627,7 @@
         </is>
       </c>
       <c r="N72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O72" t="inlineStr">
         <is>
@@ -18651,7 +18651,7 @@
         </is>
       </c>
       <c r="T72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73">
@@ -18857,7 +18857,7 @@
         </is>
       </c>
       <c r="J75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -21235,7 +21235,7 @@
         </is>
       </c>
       <c r="N104" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O104" t="inlineStr">
         <is>
@@ -21465,7 +21465,7 @@
         </is>
       </c>
       <c r="J107" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K107" t="inlineStr">
         <is>
@@ -22827,7 +22827,7 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G124" t="inlineStr">
         <is>
@@ -22863,7 +22863,7 @@
         </is>
       </c>
       <c r="P124" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q124" t="inlineStr">
         <is>
@@ -23307,7 +23307,7 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
@@ -23815,7 +23815,7 @@
         </is>
       </c>
       <c r="L136" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M136" t="inlineStr">
         <is>
@@ -24029,7 +24029,7 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G139" t="inlineStr">
         <is>
@@ -24423,7 +24423,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -24513,7 +24513,7 @@
         </is>
       </c>
       <c r="F145" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G145" t="inlineStr">
         <is>
@@ -24529,7 +24529,7 @@
         </is>
       </c>
       <c r="J145" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K145" t="inlineStr">
         <is>
@@ -24537,7 +24537,7 @@
         </is>
       </c>
       <c r="L145" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M145" t="inlineStr">
         <is>
@@ -24713,7 +24713,7 @@
         </is>
       </c>
       <c r="R147" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S147" t="inlineStr">
         <is>
@@ -24821,7 +24821,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -24837,7 +24837,7 @@
         </is>
       </c>
       <c r="H149" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I149" t="inlineStr">
         <is>
@@ -24857,7 +24857,7 @@
         </is>
       </c>
       <c r="N149" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O149" t="inlineStr"/>
       <c r="P149" t="n">
@@ -26071,7 +26071,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -26087,7 +26087,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -26111,7 +26111,7 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -26119,7 +26119,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -26625,7 +26625,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -26985,7 +26985,7 @@
         </is>
       </c>
       <c r="T25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
@@ -27155,7 +27155,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -27245,7 +27245,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -27253,7 +27253,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -27269,7 +27269,7 @@
         </is>
       </c>
       <c r="L29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
@@ -27277,7 +27277,7 @@
         </is>
       </c>
       <c r="N29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -27301,7 +27301,7 @@
         </is>
       </c>
       <c r="T29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -27553,7 +27553,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -27577,7 +27577,7 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -27593,7 +27593,7 @@
         </is>
       </c>
       <c r="N33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -27609,7 +27609,7 @@
         </is>
       </c>
       <c r="R33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S33" t="inlineStr">
         <is>
@@ -29909,7 +29909,7 @@
         </is>
       </c>
       <c r="J63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
@@ -30479,7 +30479,7 @@
         </is>
       </c>
       <c r="P70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q70" t="inlineStr">
         <is>
@@ -30779,7 +30779,7 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -31079,7 +31079,7 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -31119,7 +31119,7 @@
         </is>
       </c>
       <c r="P78" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q78" t="inlineStr">
         <is>
@@ -31135,7 +31135,7 @@
         </is>
       </c>
       <c r="T78" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79">
@@ -32213,7 +32213,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -32229,7 +32229,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
@@ -32237,7 +32237,7 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -32253,7 +32253,7 @@
         </is>
       </c>
       <c r="N93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
@@ -32277,7 +32277,7 @@
         </is>
       </c>
       <c r="T93" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
@@ -32513,7 +32513,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -32537,7 +32537,7 @@
         </is>
       </c>
       <c r="J97" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K97" t="inlineStr">
         <is>
@@ -32553,7 +32553,7 @@
         </is>
       </c>
       <c r="N97" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -33149,7 +33149,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -33629,7 +33629,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -33669,7 +33669,7 @@
         </is>
       </c>
       <c r="N111" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -33693,7 +33693,7 @@
         </is>
       </c>
       <c r="T111" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="112">
@@ -33711,7 +33711,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -33735,7 +33735,7 @@
         </is>
       </c>
       <c r="J112" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K112" t="inlineStr">
         <is>
@@ -33775,7 +33775,7 @@
         </is>
       </c>
       <c r="T112" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="113">
@@ -33793,7 +33793,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -33801,7 +33801,7 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
@@ -33833,7 +33833,7 @@
         </is>
       </c>
       <c r="N113" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -33841,7 +33841,7 @@
         </is>
       </c>
       <c r="P113" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q113" t="inlineStr">
         <is>
@@ -33849,7 +33849,7 @@
         </is>
       </c>
       <c r="R113" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S113" t="inlineStr">
         <is>
@@ -34191,7 +34191,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
@@ -34487,7 +34487,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -34503,7 +34503,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
@@ -34527,7 +34527,7 @@
         </is>
       </c>
       <c r="N122" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -34535,7 +34535,7 @@
         </is>
       </c>
       <c r="P122" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q122" t="inlineStr">
         <is>
@@ -34577,7 +34577,7 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G123" t="inlineStr"/>
       <c r="H123" t="n">
@@ -34691,7 +34691,7 @@
         </is>
       </c>
       <c r="P124" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q124" t="inlineStr">
         <is>
@@ -34699,7 +34699,7 @@
         </is>
       </c>
       <c r="R124" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S124" t="inlineStr">
         <is>
@@ -34827,7 +34827,7 @@
         </is>
       </c>
       <c r="P126" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q126" t="inlineStr">
         <is>
@@ -34835,7 +34835,7 @@
         </is>
       </c>
       <c r="R126" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S126" t="inlineStr">
         <is>
@@ -35058,7 +35058,7 @@
         </is>
       </c>
       <c r="P129" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q129" t="inlineStr">
         <is>
@@ -35066,7 +35066,7 @@
         </is>
       </c>
       <c r="R129" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S129" t="inlineStr">
         <is>
@@ -35174,7 +35174,7 @@
         </is>
       </c>
       <c r="D131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -35182,7 +35182,7 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G131" t="inlineStr">
         <is>
@@ -35198,7 +35198,7 @@
         </is>
       </c>
       <c r="J131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K131" t="inlineStr">
         <is>
@@ -35206,7 +35206,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M131" t="inlineStr">
         <is>
@@ -35222,7 +35222,7 @@
         </is>
       </c>
       <c r="P131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q131" t="inlineStr">
         <is>
@@ -35230,7 +35230,7 @@
         </is>
       </c>
       <c r="R131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S131" t="inlineStr">
         <is>
@@ -35238,7 +35238,7 @@
         </is>
       </c>
       <c r="T131" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="132">
@@ -35338,7 +35338,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -35346,7 +35346,7 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G133" t="inlineStr"/>
       <c r="H133" t="n">
@@ -35358,7 +35358,7 @@
         </is>
       </c>
       <c r="J133" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K133" t="inlineStr">
         <is>
@@ -35374,7 +35374,7 @@
         </is>
       </c>
       <c r="N133" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -35382,7 +35382,7 @@
         </is>
       </c>
       <c r="P133" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
@@ -35390,7 +35390,7 @@
         </is>
       </c>
       <c r="R133" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S133" t="inlineStr">
         <is>
@@ -35398,7 +35398,7 @@
         </is>
       </c>
       <c r="T133" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="134">
@@ -35744,7 +35744,7 @@
         </is>
       </c>
       <c r="P138" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q138" t="inlineStr">
         <is>
@@ -35752,7 +35752,7 @@
         </is>
       </c>
       <c r="R138" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S138" t="inlineStr"/>
       <c r="T138" t="n">
@@ -36110,7 +36110,7 @@
         </is>
       </c>
       <c r="J143" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K143" t="inlineStr"/>
       <c r="L143" t="n">
@@ -36126,7 +36126,7 @@
         </is>
       </c>
       <c r="P143" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q143" t="inlineStr">
         <is>
@@ -36212,7 +36212,7 @@
         </is>
       </c>
       <c r="R144" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S144" t="inlineStr">
         <is>
@@ -36494,7 +36494,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -36580,7 +36580,7 @@
         </is>
       </c>
       <c r="F150" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
@@ -36596,7 +36596,7 @@
         </is>
       </c>
       <c r="J150" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K150" t="inlineStr">
         <is>
@@ -36628,7 +36628,7 @@
         </is>
       </c>
       <c r="R150" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S150" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
update evals with FT+QSP
</commit_message>
<xml_diff>
--- a/eval/error_analysis/results/analysis_by_qid_full150.xlsx
+++ b/eval/error_analysis/results/analysis_by_qid_full150.xlsx
@@ -22819,7 +22819,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -24181,7 +24181,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -26071,7 +26071,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -26087,7 +26087,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -26111,7 +26111,7 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -26119,7 +26119,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -26625,7 +26625,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -27219,7 +27219,7 @@
         </is>
       </c>
       <c r="T28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -27245,7 +27245,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -27253,7 +27253,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -27269,7 +27269,7 @@
         </is>
       </c>
       <c r="L29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
@@ -27277,7 +27277,7 @@
         </is>
       </c>
       <c r="N29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -27301,7 +27301,7 @@
         </is>
       </c>
       <c r="T29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
@@ -27553,7 +27553,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -27577,7 +27577,7 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
@@ -27593,7 +27593,7 @@
         </is>
       </c>
       <c r="N33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -27609,7 +27609,7 @@
         </is>
       </c>
       <c r="R33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S33" t="inlineStr">
         <is>
@@ -29941,7 +29941,7 @@
         </is>
       </c>
       <c r="R63" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S63" t="inlineStr">
         <is>
@@ -30779,7 +30779,7 @@
         </is>
       </c>
       <c r="J74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K74" t="inlineStr">
         <is>
@@ -32213,7 +32213,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -32229,7 +32229,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I93" t="inlineStr">
         <is>
@@ -32237,7 +32237,7 @@
         </is>
       </c>
       <c r="J93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
@@ -32253,7 +32253,7 @@
         </is>
       </c>
       <c r="N93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O93" t="inlineStr">
         <is>
@@ -32277,7 +32277,7 @@
         </is>
       </c>
       <c r="T93" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94">
@@ -32513,7 +32513,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -32537,7 +32537,7 @@
         </is>
       </c>
       <c r="J97" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K97" t="inlineStr">
         <is>
@@ -32553,7 +32553,7 @@
         </is>
       </c>
       <c r="N97" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O97" t="inlineStr">
         <is>
@@ -33149,7 +33149,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -33629,7 +33629,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -33669,7 +33669,7 @@
         </is>
       </c>
       <c r="N111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>
@@ -33693,7 +33693,7 @@
         </is>
       </c>
       <c r="T111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="112">
@@ -33711,7 +33711,7 @@
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -33775,7 +33775,7 @@
         </is>
       </c>
       <c r="T112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113">
@@ -33793,7 +33793,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -33833,7 +33833,7 @@
         </is>
       </c>
       <c r="N113" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O113" t="inlineStr">
         <is>
@@ -33841,7 +33841,7 @@
         </is>
       </c>
       <c r="P113" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q113" t="inlineStr">
         <is>
@@ -34191,7 +34191,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I118" t="inlineStr">
         <is>
@@ -34503,7 +34503,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I122" t="inlineStr">
         <is>
@@ -34527,7 +34527,7 @@
         </is>
       </c>
       <c r="N122" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O122" t="inlineStr">
         <is>
@@ -34535,7 +34535,7 @@
         </is>
       </c>
       <c r="P122" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q122" t="inlineStr">
         <is>
@@ -35100,7 +35100,7 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
@@ -35374,7 +35374,7 @@
         </is>
       </c>
       <c r="N133" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O133" t="inlineStr">
         <is>
@@ -35382,7 +35382,7 @@
         </is>
       </c>
       <c r="P133" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q133" t="inlineStr">
         <is>
@@ -35390,7 +35390,7 @@
         </is>
       </c>
       <c r="R133" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S133" t="inlineStr">
         <is>
@@ -35398,7 +35398,7 @@
         </is>
       </c>
       <c r="T133" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="134">
@@ -35744,7 +35744,7 @@
         </is>
       </c>
       <c r="P138" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q138" t="inlineStr">
         <is>
@@ -35752,7 +35752,7 @@
         </is>
       </c>
       <c r="R138" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S138" t="inlineStr"/>
       <c r="T138" t="n">
@@ -36110,7 +36110,7 @@
         </is>
       </c>
       <c r="J143" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K143" t="inlineStr"/>
       <c r="L143" t="n">
@@ -36126,7 +36126,7 @@
         </is>
       </c>
       <c r="P143" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q143" t="inlineStr">
         <is>
@@ -36596,7 +36596,7 @@
         </is>
       </c>
       <c r="J150" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K150" t="inlineStr">
         <is>
@@ -36628,7 +36628,7 @@
         </is>
       </c>
       <c r="R150" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S150" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
add precision and recall by qid
</commit_message>
<xml_diff>
--- a/eval/error_analysis/results/analysis_by_qid_full150.xlsx
+++ b/eval/error_analysis/results/analysis_by_qid_full150.xlsx
@@ -19472,7 +19472,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>RT, IN</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -19481,7 +19481,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -19489,7 +19489,7 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G83" t="inlineStr">
         <is>
@@ -19497,7 +19497,7 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
@@ -19505,7 +19505,7 @@
         </is>
       </c>
       <c r="J83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K83" t="inlineStr">
         <is>
@@ -19513,7 +19513,7 @@
         </is>
       </c>
       <c r="L83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M83" t="inlineStr">
         <is>
@@ -19521,7 +19521,7 @@
         </is>
       </c>
       <c r="N83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O83" t="inlineStr">
         <is>
@@ -19529,7 +19529,7 @@
         </is>
       </c>
       <c r="P83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q83" t="inlineStr">
         <is>
@@ -19537,7 +19537,7 @@
         </is>
       </c>
       <c r="R83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S83" t="inlineStr">
         <is>
@@ -19545,7 +19545,7 @@
         </is>
       </c>
       <c r="T83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84">
@@ -21752,7 +21752,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>PR, RT, IN</t>
+          <t>IN</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -21769,7 +21769,7 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
@@ -21801,7 +21801,7 @@
         </is>
       </c>
       <c r="N111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
exact vs partial -- list type metrics
</commit_message>
<xml_diff>
--- a/eval/error_analysis/results/analysis_by_qid_full150.xlsx
+++ b/eval/error_analysis/results/analysis_by_qid_full150.xlsx
@@ -21752,56 +21752,56 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
+          <t>PR, RT, IN</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>0</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D111" t="n">
-        <v>0</v>
-      </c>
-      <c r="E111" t="inlineStr">
+      <c r="F111" t="n">
+        <v>0</v>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Not reported</t>
+        </is>
+      </c>
+      <c r="H111" t="n">
+        <v>0</v>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J111" t="n">
+        <v>0</v>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L111" t="n">
+        <v>0</v>
+      </c>
+      <c r="M111" t="inlineStr">
         <is>
           <t>IN</t>
         </is>
       </c>
-      <c r="F111" t="n">
-        <v>1</v>
-      </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="H111" t="n">
-        <v>0</v>
-      </c>
-      <c r="I111" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="J111" t="n">
-        <v>0</v>
-      </c>
-      <c r="K111" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="L111" t="n">
-        <v>0</v>
-      </c>
-      <c r="M111" t="inlineStr">
-        <is>
-          <t>IN</t>
-        </is>
-      </c>
       <c r="N111" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O111" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
generate figures by using new eval algorithm
</commit_message>
<xml_diff>
--- a/eval/error_analysis/results/analysis_by_qid_full150.xlsx
+++ b/eval/error_analysis/results/analysis_by_qid_full150.xlsx
@@ -16679,7 +16679,7 @@
         </is>
       </c>
       <c r="P48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q48" t="inlineStr">
         <is>
@@ -18857,7 +18857,7 @@
         </is>
       </c>
       <c r="J75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K75" t="inlineStr">
         <is>
@@ -21465,7 +21465,7 @@
         </is>
       </c>
       <c r="J107" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K107" t="inlineStr">
         <is>
@@ -22819,7 +22819,7 @@
         </is>
       </c>
       <c r="D124" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -22827,7 +22827,7 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G124" t="inlineStr">
         <is>
@@ -22863,7 +22863,7 @@
         </is>
       </c>
       <c r="P124" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q124" t="inlineStr">
         <is>
@@ -24829,7 +24829,7 @@
         </is>
       </c>
       <c r="F149" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G149" t="inlineStr">
         <is>

</xml_diff>